<commit_message>
docs(planning): add implementer + reviewer effort columns
Adds two t-shirt-sized effort columns (XS / S / M / L / XL, mapped to
Claude Code session-hour ranges) per phase, with reasoning extended to
explain the size. Effort × model rate gives the cost-estimate signal
the matrix was missing in the first cut.

Legend sheet documents the size scale and adds the 25-35% reviewer-vs-
implementer-effort heuristic.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/spreadsheet/phase_model_plan.xlsx
+++ b/docs/spreadsheet/phase_model_plan.xlsx
@@ -39,7 +39,7 @@
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -58,12 +58,37 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EAF3FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE5CD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4CCCC"/>
       </patternFill>
     </fill>
   </fills>
@@ -79,22 +104,37 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -465,17 +505,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
     <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="90" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="88" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Phase</t>
@@ -493,16 +535,26 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Implementer effort</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Reviewer model</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Reviewer effort</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Reasoning</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="100" customHeight="1">
+    <row r="2" ht="120" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Plan 1A — Foundation Setup</t>
@@ -520,16 +572,26 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
+          <t>M (4-8h)</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
           <t>Opus</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Foundation work: aiosqlite migration for the user_preferences table, JWT role-claim parsing, design-token CSS, prefs server module + endpoints. Schema and auth-claim mistakes are expensive to undo once data lands, so spend once on Opus review even though Sonnet handles the implementation comfortably.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="100" customHeight="1">
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>S (2-3h)</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Foundation work: aiosqlite migration for the user_preferences table, JWT role-claim parsing, design-token CSS, prefs server module + endpoints. Schema and auth-claim mistakes are expensive to undo once data lands, so spend once on Opus review even though Sonnet handles the implementation comfortably. Effort is medium because the scope is wide but each piece is well-defined; reviewer focuses on the migration and JWT slice (the irreversible bits), not the CSS tokens.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="120" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Plan 1B — Static Chrome</t>
@@ -540,23 +602,33 @@
           <t>2026-04-28-ux-overhaul-static-chrome.md</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>Haiku</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>S (2-4h)</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>Haiku</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Four pure-presentational vanilla-JS components (top-nav, version-chip, avatar, layout-icon), each ≤100 LOC, no state, no async, no server interaction. Pattern is repetitive and the safe-DOM rules are explicit. Cheapest tier on both sides; the review just spot-checks for innerHTML and pattern adherence.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="100" customHeight="1">
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>XS (&lt;1h)</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Four pure-presentational vanilla-JS components (top-nav, version-chip, avatar, layout-icon), each ≤100 LOC, no state, no async, no server interaction. Pattern is repetitive and the safe-DOM rules are explicit. Cheapest tier on both sides; the review just spot-checks for innerHTML and pattern adherence — fits in one short pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="120" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Plan 1C — Stateful Chrome</t>
@@ -572,18 +644,28 @@
           <t>Sonnet</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Sonnet</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Prefs client (localStorage cache + 500ms debounced PUT), telemetry helper (fire-and-forget), avatar/layout popovers with click-outside + Escape. Subtle async + event-lifecycle but well-bounded. Sonnet/Sonnet — popover bugs are visible and easy to spot at this tier; Opus is overkill.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="100" customHeight="1">
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>M (4-8h)</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>S (2-3h)</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Prefs client (localStorage cache + 500ms debounced PUT), telemetry helper (fire-and-forget), avatar/layout popovers with click-outside + Escape. Subtle async + event-lifecycle but well-bounded. Reviewer needs to follow the popover state machine + debounce semantics, hence S not XS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="120" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Plan 2A — Document Card + Density Modes</t>
@@ -594,23 +676,33 @@
           <t>2026-04-28-ux-overhaul-document-card.md</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>Haiku</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Sonnet</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Presentational card component with three density modes driven by CSS variables and MFPrefs. Implementation is mechanical given the explicit mockups, but bumping reviewer to Sonnet because density toggle interacts with the prefs system landed in 1C — worth verifying the binding is correct, not just the visuals.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="100" customHeight="1">
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>S (2-4h)</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>XS (&lt;1h)</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Presentational card component with three density modes driven by CSS variables and MFPrefs. Implementation is mechanical given the explicit mockups, but bumping reviewer to Sonnet because density toggle interacts with the prefs system landed in 1C — worth verifying the binding is correct, not just the visuals. Review fits in a single short pass since the surface area is small.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="120" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Plan 2B — Card Interactions</t>
@@ -626,18 +718,28 @@
           <t>Sonnet</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>Sonnet</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Hover preview popover, right-click context menu, multi-select observable state, bulk action bar, folder-browse page wrapping it all. Multiple interaction systems coexisting without listener leaks is the failure mode here. Sonnet handles the orchestration; Sonnet review catches missed cleanup paths.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="100" customHeight="1">
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>L (8-16h)</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>M (3-5h)</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Hover preview popover, right-click context menu, multi-select observable state, bulk action bar, folder-browse page wrapping it all. Multiple interaction systems coexisting without listener leaks is the failure mode. This is the biggest UX-overhaul phase — reviewer needs M because there are 4 distinct interaction surfaces to walk through, not one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="120" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Plan 3 — Search-as-Home Page</t>
@@ -653,18 +755,28 @@
           <t>Sonnet</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>Sonnet</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Feature-flagged replacement of static/index.html with three layout modes (Maximal / Recent / Minimal). Both flag-on and flag-off paths must work — flag-off keeps legacy Convert page live, so rollback is cheap. Not security-critical, doesn't touch DB or auth, so Sonnet/Sonnet is the right floor.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="100" customHeight="1">
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>M (4-8h)</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>S (2-3h)</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Feature-flagged replacement of static/index.html with three layout modes (Maximal / Recent / Minimal). Both flag-on and flag-off paths must work — flag-off keeps legacy Convert page live, so rollback is cheap. Reviewer's main job is verifying the flag branching and that legacy still renders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="120" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Plan 4 — IA Shift</t>
@@ -682,12 +794,22 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
+          <t>M (4-8h)</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
           <t>Opus</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>New /api/me endpoint, real role binding via UnionCore JWT (replaces the hardcoded role='admin' placeholder), Activity dashboard gated by core.auth.Role. This is the auth surface — role-gating bugs are security issues. Opus reviewer once to verify the gate is enforced on every protected endpoint, not just the obvious ones.</t>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>S (2-3h)</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>New /api/me endpoint, real role binding via UnionCore JWT (replaces the hardcoded role='admin' placeholder), Activity dashboard gated by core.auth.Role. Auth surface — role-gating bugs are security issues. Opus reviewer once to verify the gate is enforced on every protected endpoint, not just the obvious ones; effort is small because the new endpoint surface is narrow.</t>
         </is>
       </c>
     </row>
@@ -702,17 +824,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:G7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
     <col width="48" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="90" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="88" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Phase</t>
@@ -730,16 +854,26 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Implementer effort</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Reviewer model</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Reviewer effort</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Reasoning</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="100" customHeight="1">
+    <row r="2" ht="120" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Phase 0 — Pre-flight reconnaissance (Tasks 0.1–0.7)</t>
@@ -750,23 +884,33 @@
           <t>2026-04-28-active-operations-registry.md</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>Haiku</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
+        <is>
+          <t>S (2-4h)</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>Haiku</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Read-only discovery: trace existing pipeline.py, scan_coordinator.py, bulk_worker.py, lifecycle_scanner.py to confirm assumptions about cancel signals and lifecycle hooks. Output is notes, not code. Cheapest tier on both sides; Haiku is good enough for summarising existing module behaviour against the plan's assumptions.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="100" customHeight="1">
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>XS (&lt;1h)</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Read-only discovery: trace existing pipeline.py, scan_coordinator.py, bulk_worker.py, lifecycle_scanner.py to confirm assumptions about cancel signals and lifecycle hooks. Output is notes, not code. Cheapest tier on both sides; review is just a sanity-check that the recon notes match the plan's stated assumptions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="120" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Phase 1 — Registry + DB foundation (Tasks 1–10)</t>
@@ -777,23 +921,33 @@
           <t>2026-04-28-active-operations-registry.md</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>Opus</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>L (8-16h)</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>Opus</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Load-bearing concurrency primitive: new core/active_ops.py (in-memory dict + write-through to a new active_operations SQLite table), lifespan hooks, scheduler integration, singleton lifecycle. Every later phase depends on this being correct — race conditions or write-through gaps cascade across all six worker subsystems. Spend tokens here; it is genuinely the highest-risk slice of the whole plan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="100" customHeight="1">
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>M (3-5h)</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Load-bearing concurrency primitive: new core/active_ops.py (in-memory dict + write-through to a new active_operations SQLite table), lifespan hooks, scheduler integration, singleton lifecycle. Every later phase depends on this — race conditions or write-through gaps cascade across all six worker subsystems. Spend tokens here on both sides; this is the genuinely highest-risk slice of the whole plan and the only place where Opus/Opus is unconditionally the right call.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="120" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Phase 2 — HTTP API (Tasks 11–13)</t>
@@ -809,18 +963,28 @@
           <t>Sonnet</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>Sonnet</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>Single GET /api/active-ops endpoint feeding three frontend surfaces. Standard FastAPI pattern with a strict response schema. Risk is contract drift between this payload and Phase 4's three consumers — Sonnet reviewer is sufficient because the payload is small and reviewable in one screen.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="100" customHeight="1">
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>S (2-4h)</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>XS (&lt;1h)</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Single GET /api/active-ops endpoint feeding three frontend surfaces. Standard FastAPI pattern with a strict response schema. Review is a quick contract check against Phase 4's three consumers; payload is small and readable in one screen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="120" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Phase 3 — Worker retrofits (Tasks 14–23)</t>
@@ -831,23 +995,33 @@
           <t>2026-04-28-active-operations-registry.md</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>Opus</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
-        <is>
-          <t>Sonnet</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Touches six worker modules (pipeline, scan_coordinator, trash, analysis, lifecycle_scanner, bulk_worker) to register/update/finish operations and bridge cancel signals to each subsystem's native mechanism. The structural traps — double-register, missed cleanup on exception paths, cancel hook never firing — need Opus to catch on the implementer side. Reviewer drops to Sonnet to control cost; the implementer does the heavy thinking.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="100" customHeight="1">
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>XL (16-32h)</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr">
+        <is>
+          <t>L (5-8h)</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Touches six worker modules (pipeline, scan_coordinator, trash, analysis, lifecycle_scanner, bulk_worker) to register/update/finish operations and bridge cancel signals to each subsystem's native mechanism. Largest phase by far. The structural traps — double-register, missed cleanup on exception paths, cancel hook never firing — need Opus to catch on the implementer side. Reviewer at Sonnet has 6 modules × cancel paths to walk through, hence L not M.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="120" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Phase 4 — Frontend (Tasks 24–34)</t>
@@ -863,18 +1037,28 @@
           <t>Sonnet</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>L (8-16h)</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
         <is>
           <t>Haiku</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Three presentational surfaces (sticky banner, per-page inline widget, Status hub) all fed by the /api/active-ops payload from Phase 2. Once that contract is stable the work is mechanical DOM construction + polling. Haiku reviewer is fine — visual diff against mockups is exactly what cheap models do well.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="100" customHeight="1">
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>S (2-3h)</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Three presentational surfaces (sticky banner, per-page inline widget, Status hub) all fed by the /api/active-ops payload from Phase 2. 11 tasks across the three surfaces. Once that contract is stable the work is mechanical DOM construction + polling. Haiku reviewer is fine — visual diff against mockups is exactly what cheap models do well — but they need S not XS because there are three surfaces to compare.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="120" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Phase 5 — Cleanup + documentation (Tasks 35–46)</t>
@@ -890,14 +1074,24 @@
           <t>Sonnet</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
-        <is>
-          <t>Sonnet</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Removing dead per-subsystem progress code that the registry now subsumes, plus CLAUDE.md / version-history.md / whats-new.md updates. Deletions are irreversible — judgement about what's truly subsumed vs. what still has unique callers needs Sonnet, not Haiku. Sonnet reviewer catches the cases where the implementer was over-eager.</t>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>M (4-8h)</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>S (2-3h)</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Removing dead per-subsystem progress code that the registry now subsumes, plus CLAUDE.md / version-history.md / whats-new.md updates. 12 tasks. Deletions are irreversible — judgement about what's truly subsumed vs. what still has unique callers needs Sonnet, not Haiku. Reviewer focus is on the deletions, not the doc edits.</t>
         </is>
       </c>
     </row>
@@ -912,7 +1106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -921,30 +1115,30 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Model legend &amp; cost guidance</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="12" t="inlineStr">
         <is>
           <t>Use for</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="12" t="inlineStr">
         <is>
           <t>Approx cost vs Opus</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="50" customHeight="1">
+    <row r="4" ht="38" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Haiku</t>
@@ -961,7 +1155,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="50" customHeight="1">
+    <row r="5" ht="38" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Sonnet</t>
@@ -978,7 +1172,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="50" customHeight="1">
+    <row r="6" ht="38" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Opus</t>
@@ -995,23 +1189,106 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="50" customHeight="1">
+    <row r="7" ht="38" customHeight="1">
       <c r="A7" s="2" t="inlineStr"/>
       <c r="B7" s="2" t="inlineStr"/>
       <c r="C7" s="2" t="inlineStr"/>
     </row>
-    <row r="8" ht="50" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="8" ht="38" customHeight="1">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Effort size</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>Approx Claude Code session-hours</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9" ht="38" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>&lt;2h — single short pass; cosmetic edits, narrow contract checks.</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10" ht="38" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>2-4h — one focused session.</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11" ht="38" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>4-8h — half-day to a day; multi-file feature.</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12" ht="38" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>8-16h — one to two days; multiple interacting components.</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13" ht="38" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>16-32h — multi-day; touches several subsystems (e.g. Phase 3 worker retrofits).</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14" ht="38" customHeight="1">
+      <c r="A14" s="2" t="inlineStr"/>
+      <c r="B14" s="2" t="inlineStr"/>
+      <c r="C14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15" ht="38" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>Heuristic</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Default both implementer and reviewer to Sonnet. Justify every upgrade to Opus (irreversibility, security, concurrency) and every downgrade to Haiku (mechanical, well-spec'd, low blast radius).</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr"/>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Default both implementer and reviewer to Sonnet/M. Justify every Opus upgrade (irreversibility, security, concurrency) and every Haiku downgrade (mechanical, well-spec'd, low blast radius). Reviewer effort runs ~25-35% of implementer effort for a single focused pass — bigger if the implementer touched many subsystems.</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs(planning): use Claude low/med/high/max syntax for effort scale
Replaces XS/S/M/L/XL labels with Claude Code's native low/med/high/max
thinking-budget vocabulary so the effort column reads consistently with
how Claude Code session sizing is talked about elsewhere. Hour ranges
preserved in parentheses for cost math.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/spreadsheet/phase_model_plan.xlsx
+++ b/docs/spreadsheet/phase_model_plan.xlsx
@@ -39,7 +39,7 @@
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -78,11 +78,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EAF3FB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00FCE5CD"/>
       </patternFill>
     </fill>
@@ -104,7 +99,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -131,9 +126,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -572,7 +564,7 @@
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>M (4-8h)</t>
+          <t>med (4-8h)</t>
         </is>
       </c>
       <c r="E2" s="5" t="inlineStr">
@@ -582,7 +574,7 @@
       </c>
       <c r="F2" s="6" t="inlineStr">
         <is>
-          <t>S (2-3h)</t>
+          <t>low (2-3h)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -609,7 +601,7 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>S (2-4h)</t>
+          <t>low (2-4h)</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
@@ -617,9 +609,9 @@
           <t>Haiku</t>
         </is>
       </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>XS (&lt;1h)</t>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>low (&lt;1h)</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -646,7 +638,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>M (4-8h)</t>
+          <t>med (4-8h)</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -656,7 +648,7 @@
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>S (2-3h)</t>
+          <t>low (2-3h)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -683,7 +675,7 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>S (2-4h)</t>
+          <t>low (2-4h)</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -691,9 +683,9 @@
           <t>Sonnet</t>
         </is>
       </c>
-      <c r="F5" s="8" t="inlineStr">
-        <is>
-          <t>XS (&lt;1h)</t>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>low (&lt;1h)</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -718,9 +710,9 @@
           <t>Sonnet</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>L (8-16h)</t>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>high (8-16h)</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -730,7 +722,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>M (3-5h)</t>
+          <t>med (3-5h)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -757,7 +749,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>M (4-8h)</t>
+          <t>med (4-8h)</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -767,7 +759,7 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>S (2-3h)</t>
+          <t>low (2-3h)</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -794,7 +786,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>M (4-8h)</t>
+          <t>med (4-8h)</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -804,7 +796,7 @@
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>S (2-3h)</t>
+          <t>low (2-3h)</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -891,7 +883,7 @@
       </c>
       <c r="D2" s="6" t="inlineStr">
         <is>
-          <t>S (2-4h)</t>
+          <t>low (2-4h)</t>
         </is>
       </c>
       <c r="E2" s="7" t="inlineStr">
@@ -899,9 +891,9 @@
           <t>Haiku</t>
         </is>
       </c>
-      <c r="F2" s="8" t="inlineStr">
-        <is>
-          <t>XS (&lt;1h)</t>
+      <c r="F2" s="6" t="inlineStr">
+        <is>
+          <t>low (&lt;1h)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -926,9 +918,9 @@
           <t>Opus</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
-        <is>
-          <t>L (8-16h)</t>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>high (8-16h)</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -938,7 +930,7 @@
       </c>
       <c r="F3" s="4" t="inlineStr">
         <is>
-          <t>M (3-5h)</t>
+          <t>med (3-5h)</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -965,7 +957,7 @@
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>S (2-4h)</t>
+          <t>low (2-4h)</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -973,9 +965,9 @@
           <t>Sonnet</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>XS (&lt;1h)</t>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>low (&lt;1h)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1000,9 +992,9 @@
           <t>Opus</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr">
-        <is>
-          <t>XL (16-32h)</t>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
+          <t>max (16-32h)</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -1010,9 +1002,9 @@
           <t>Sonnet</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
-        <is>
-          <t>L (5-8h)</t>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>med (5-8h)</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -1037,9 +1029,9 @@
           <t>Sonnet</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>L (8-16h)</t>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>high (8-16h)</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
@@ -1049,7 +1041,7 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>S (2-3h)</t>
+          <t>low (2-3h)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1076,7 +1068,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>M (4-8h)</t>
+          <t>med (4-8h)</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -1086,7 +1078,7 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>S (2-3h)</t>
+          <t>low (2-3h)</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -1106,7 +1098,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C15"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1115,24 +1107,24 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="11" t="inlineStr">
+      <c r="A1" s="10" t="inlineStr">
         <is>
           <t>Model legend &amp; cost guidance</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="B3" s="12" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Use for</t>
         </is>
       </c>
-      <c r="C3" s="12" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>Approx cost vs Opus</t>
         </is>
@@ -1195,14 +1187,14 @@
       <c r="C7" s="2" t="inlineStr"/>
     </row>
     <row r="8" ht="38" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>Effort size</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t>Approx Claude Code session-hours</t>
+      <c r="A8" s="11" t="inlineStr">
+        <is>
+          <t>Effort</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Claude Code session-hours (label matches Claude's low/med/high/max thinking-budget syntax)</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr"/>
@@ -1210,12 +1202,12 @@
     <row r="9" ht="38" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>XS</t>
+          <t>low</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>&lt;2h — single short pass; cosmetic edits, narrow contract checks.</t>
+          <t>&lt;4h — short pass; small contract checks, scaffold components, recon notes.</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr"/>
@@ -1223,12 +1215,12 @@
     <row r="10" ht="38" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>med</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>2-4h — one focused session.</t>
+          <t>4-8h — half-day to a day; multi-file feature, focused review of a critical slice.</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr"/>
@@ -1236,12 +1228,12 @@
     <row r="11" ht="38" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>high</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>4-8h — half-day to a day; multi-file feature.</t>
+          <t>8-16h — one to two days; multiple interacting components or subsystem-spanning review.</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr"/>
@@ -1249,46 +1241,33 @@
     <row r="12" ht="38" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>max</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>8-16h — one to two days; multiple interacting components.</t>
+          <t>16-32h — multi-day; touches several subsystems (e.g. Active-Ops Phase 3 worker retrofits).</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr"/>
     </row>
     <row r="13" ht="38" customHeight="1">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>XL</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>16-32h — multi-day; touches several subsystems (e.g. Phase 3 worker retrofits).</t>
-        </is>
-      </c>
+      <c r="A13" s="2" t="inlineStr"/>
+      <c r="B13" s="2" t="inlineStr"/>
       <c r="C13" s="2" t="inlineStr"/>
     </row>
     <row r="14" ht="38" customHeight="1">
-      <c r="A14" s="2" t="inlineStr"/>
-      <c r="B14" s="2" t="inlineStr"/>
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Heuristic</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Default both implementer and reviewer to Sonnet at med. Justify every Opus upgrade (irreversibility, security, concurrency) and every Haiku downgrade (mechanical, well-spec'd, low blast radius). Reviewer effort runs ~25-35% of implementer effort for a single focused pass — bigger if the implementer touched many subsystems.</t>
+        </is>
+      </c>
       <c r="C14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15" ht="38" customHeight="1">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Heuristic</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Default both implementer and reviewer to Sonnet/M. Justify every Opus upgrade (irreversibility, security, concurrency) and every Haiku downgrade (mechanical, well-spec'd, low blast radius). Reviewer effort runs ~25-35% of implementer effort for a single focused pass — bigger if the implementer touched many subsystems.</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>